<commit_message>
Correct MotivateToSeattle's dance schedule data
Replace placeholder "Various" levels with the actual scheduled levels
for GCA Callers/Trail-In Dance (Friday) and Closing (Sunday); move
Registration and Brunch into the Lobby room instead of an early-morning
roomless note and an all-rooms span, respectively; simplify Columbia's
C3A/C3B block to C3A alone (C3A/C4 on Sunday afternoon).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10802"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB82C6B-4DDA-D14A-B915-90FDFC4EB93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880466E4-CE12-4741-B9C4-B6F9C4C70AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Friday October 9" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="56">
   <si>
     <t>Time</t>
   </si>
@@ -37,10 +37,6 @@
     <t>7:00p-8:00p</t>
   </si>
   <si>
-    <t>Various : Trail-In Dance - All Headliners
-ROOMS: Glacier, Horizon</t>
-  </si>
-  <si>
     <t>8:00p-9:00p</t>
   </si>
   <si>
@@ -96,9 +92,6 @@
   </si>
   <si>
     <t>A2 : Vic Ceder</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B &amp; C4 : Michael Kellogg</t>
   </si>
   <si>
     <t>12:00p-1:00p</t>
@@ -139,55 +132,64 @@
     <t>9:00a-11:00a</t>
   </si>
   <si>
-    <t>* Brunch
-ROOMS: Glacier, Horizon, Alpine, Columbia</t>
-  </si>
-  <si>
     <t>C3B : Rob French</t>
   </si>
   <si>
-    <t>Various : Closing - All Headliners
+    <t>6:30-7:00p</t>
+  </si>
+  <si>
+    <t>"</t>
+  </si>
+  <si>
+    <t>Lobby</t>
+  </si>
+  <si>
+    <t>* Registration</t>
+  </si>
+  <si>
+    <t>5:30-8:00p</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1 &amp; C2 : Trail-In Dance - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
   <si>
-    <t>6:30-7:00p</t>
-  </si>
-  <si>
-    <t>Various: GCA Callers</t>
-  </si>
-  <si>
-    <t>"</t>
-  </si>
-  <si>
-    <t>5:30-6:30</t>
-  </si>
-  <si>
-    <t>* Registration (open until 8:00 in Lobby)
-ROOMS: None</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B : Ray Brendzy</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B : Michael Kellogg</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B  : Rob French</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B  : Vic Ceder</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B  : Saundra Bryant</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B  : Ray Brendzy</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B  : Michael Kellogg</t>
-  </si>
-  <si>
-    <t>C3A &amp; C3B : Rob French</t>
+    <t>A2 &amp; C1 &amp; C2: GCA Callers</t>
+  </si>
+  <si>
+    <t>C3A   : Vic Ceder</t>
+  </si>
+  <si>
+    <t>C3A  : Rob French</t>
+  </si>
+  <si>
+    <t>C3A  : Ray Brendzy</t>
+  </si>
+  <si>
+    <t>C3A  : Michael Kellogg</t>
+  </si>
+  <si>
+    <t>C3A   : Rob French</t>
+  </si>
+  <si>
+    <t>C3A   : Saundra Bryant</t>
+  </si>
+  <si>
+    <t>C3A   : Ray Brendzy</t>
+  </si>
+  <si>
+    <t>C3A   : Michael Kellogg</t>
+  </si>
+  <si>
+    <t>C3A  &amp; C4 : Michael Kellogg</t>
+  </si>
+  <si>
+    <t>* Brunch in Lobby
+ROOMS: NONE</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1 : Closing - All Headliners
+ROOMS: Glacier, Horizon</t>
   </si>
 </sst>
 </file>
@@ -583,94 +585,102 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="5" width="30" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>43</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>54</v>
+      <c r="F6" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -707,33 +717,33 @@
     </row>
     <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>47</v>
@@ -741,16 +751,16 @@
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>48</v>
@@ -758,41 +768,41 @@
     </row>
     <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>49</v>
@@ -800,33 +810,33 @@
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>49</v>
@@ -834,10 +844,10 @@
     </row>
     <row r="10" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -845,50 +855,50 @@
         <v>5</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -899,95 +909,102 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="5" width="30" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>41</v>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
No C2 in big sessions
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10802"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880466E4-CE12-4741-B9C4-B6F9C4C70AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4434D731-5136-4542-AD5E-C063617ACD7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Friday October 9" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="55">
   <si>
     <t>Time</t>
   </si>
@@ -150,13 +150,6 @@
     <t>5:30-8:00p</t>
   </si>
   <si>
-    <t>A2 &amp; C1 &amp; C2 : Trail-In Dance - All Headliners
-ROOMS: Glacier, Horizon</t>
-  </si>
-  <si>
-    <t>A2 &amp; C1 &amp; C2: GCA Callers</t>
-  </si>
-  <si>
     <t>C3A   : Vic Ceder</t>
   </si>
   <si>
@@ -179,9 +172,6 @@
   </si>
   <si>
     <t>C3A   : Michael Kellogg</t>
-  </si>
-  <si>
-    <t>C3A  &amp; C4 : Michael Kellogg</t>
   </si>
   <si>
     <t>* Brunch in Lobby
@@ -189,6 +179,13 @@
   </si>
   <si>
     <t>A2 &amp; C1 : Closing - All Headliners
+ROOMS: Glacier, Horizon</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1: GCA Callers</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1: Trail-In Dance - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
 </sst>
@@ -630,7 +627,7 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>39</v>
@@ -644,7 +641,7 @@
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -662,7 +659,7 @@
         <v>9</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -680,7 +677,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +743,7 @@
         <v>22</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -763,7 +760,7 @@
         <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
@@ -805,7 +802,7 @@
         <v>31</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -822,7 +819,7 @@
         <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -839,7 +836,7 @@
         <v>13</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="32" x14ac:dyDescent="0.2">
@@ -864,7 +861,7 @@
         <v>17</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -881,7 +878,7 @@
         <v>22</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -898,7 +895,7 @@
         <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -941,7 +938,7 @@
         <v>36</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -977,7 +974,7 @@
         <v>17</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -995,7 +992,7 @@
         <v>31</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -1004,7 +1001,7 @@
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make the hour-tabs generator script content-set-driven
WORKBOOK_PATH was hardcoded to backtrack2abq's workbook, so it could
never target any other event. Now reads a required CONTENT_SET env
var (assertContentSetExists fails loud on a missing/mistyped value,
since this writes directly to a real spreadsheet on disk) and builds
the path from that instead. Updated docs/testing.md's usage section
to match.

Also regenerated both real events' "- Hours by Level"/"- Hours by
Caller" tabs with the current script (MotivateToSeattle for the first
time; backtrack2abq's re-run to stay consistent with the new usage).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -1,27 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10802"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4434D731-5136-4542-AD5E-C063617ACD7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Friday October 9" sheetId="1" r:id="rId1"/>
-    <sheet name="Saturday October 10" sheetId="2" r:id="rId2"/>
-    <sheet name="Sunday October 11" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Friday October 9" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Saturday October 10" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sunday October 11" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="- Hours by Level" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="- Hours by Caller" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="76">
   <si>
     <t>Time</t>
   </si>
   <si>
+    <t>Lobby</t>
+  </si>
+  <si>
     <t>Glacier</t>
   </si>
   <si>
@@ -34,9 +38,28 @@
     <t>Columbia</t>
   </si>
   <si>
+    <t>5:30-8:00p</t>
+  </si>
+  <si>
+    <t>* Registration</t>
+  </si>
+  <si>
+    <t>6:30-7:00p</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1: GCA Callers</t>
+  </si>
+  <si>
+    <t>"</t>
+  </si>
+  <si>
     <t>7:00p-8:00p</t>
   </si>
   <si>
+    <t xml:space="preserve">A2 &amp; C1: Trail-In Dance - All Headliners
+ROOMS: Glacier, Horizon</t>
+  </si>
+  <si>
     <t>8:00p-9:00p</t>
   </si>
   <si>
@@ -49,6 +72,9 @@
     <t>C2 : Rob French</t>
   </si>
   <si>
+    <t>C3A   : Vic Ceder</t>
+  </si>
+  <si>
     <t>9:00p-10:00p</t>
   </si>
   <si>
@@ -61,6 +87,9 @@
     <t>C2 : Saundra Bryant</t>
   </si>
   <si>
+    <t>C3A  : Rob French</t>
+  </si>
+  <si>
     <t>9:00a-10:00a</t>
   </si>
   <si>
@@ -88,16 +117,22 @@
     <t>C2 : Michael Kellogg</t>
   </si>
   <si>
+    <t>C3A  : Ray Brendzy</t>
+  </si>
+  <si>
     <t>11:00a-12:00p</t>
   </si>
   <si>
     <t>A2 : Vic Ceder</t>
   </si>
   <si>
+    <t>C3A  : Michael Kellogg</t>
+  </si>
+  <si>
     <t>12:00p-1:00p</t>
   </si>
   <si>
-    <t>* Lunch Break (on your own)
+    <t xml:space="preserve">* Lunch Break (on your own)
 ROOMS: NONE</t>
   </si>
   <si>
@@ -116,6 +151,9 @@
     <t>C2 : Vic Ceder</t>
   </si>
   <si>
+    <t>C3A   : Rob French</t>
+  </si>
+  <si>
     <t>3:00p-4:00p</t>
   </si>
   <si>
@@ -125,88 +163,120 @@
     <t>5:00p-7:00p</t>
   </si>
   <si>
-    <t>* Dinner Break (on your own)
+    <t xml:space="preserve">* Dinner Break (on your own)
 ROOMS: NONE</t>
   </si>
   <si>
+    <t>C3A   : Saundra Bryant</t>
+  </si>
+  <si>
+    <t>C3A   : Ray Brendzy</t>
+  </si>
+  <si>
+    <t>C3A   : Michael Kellogg</t>
+  </si>
+  <si>
     <t>9:00a-11:00a</t>
   </si>
   <si>
+    <t xml:space="preserve">* Brunch in Lobby
+ROOMS: NONE</t>
+  </si>
+  <si>
     <t>C3B : Rob French</t>
   </si>
   <si>
-    <t>6:30-7:00p</t>
-  </si>
-  <si>
-    <t>"</t>
-  </si>
-  <si>
-    <t>Lobby</t>
-  </si>
-  <si>
-    <t>* Registration</t>
-  </si>
-  <si>
-    <t>5:30-8:00p</t>
-  </si>
-  <si>
-    <t>C3A   : Vic Ceder</t>
-  </si>
-  <si>
-    <t>C3A  : Rob French</t>
-  </si>
-  <si>
-    <t>C3A  : Ray Brendzy</t>
-  </si>
-  <si>
-    <t>C3A  : Michael Kellogg</t>
-  </si>
-  <si>
-    <t>C3A   : Rob French</t>
-  </si>
-  <si>
-    <t>C3A   : Saundra Bryant</t>
-  </si>
-  <si>
-    <t>C3A   : Ray Brendzy</t>
-  </si>
-  <si>
-    <t>C3A   : Michael Kellogg</t>
-  </si>
-  <si>
-    <t>* Brunch in Lobby
-ROOMS: NONE</t>
-  </si>
-  <si>
-    <t>A2 &amp; C1 : Closing - All Headliners
+    <t xml:space="preserve">A2 &amp; C1 : Closing - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
   <si>
-    <t>A2 &amp; C1: GCA Callers</t>
-  </si>
-  <si>
-    <t>A2 &amp; C1: Trail-In Dance - All Headliners
-ROOMS: Glacier, Horizon</t>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3A</t>
+  </si>
+  <si>
+    <t>C3B</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Fri, Oct 9</t>
+  </si>
+  <si>
+    <t>Sat, Oct 10</t>
+  </si>
+  <si>
+    <t>Sun, Oct 11</t>
+  </si>
+  <si>
+    <t>Calculated</t>
+  </si>
+  <si>
+    <t>Saved</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Generated by scripts/generate-dance-schedule-hour-tabs.ts — re-run after editing any day's schedule.</t>
+  </si>
+  <si>
+    <t>Michael Kellogg</t>
+  </si>
+  <si>
+    <t>Ray Brendzy</t>
+  </si>
+  <si>
+    <t>Rob French</t>
+  </si>
+  <si>
+    <t>Saundra Bryant</t>
+  </si>
+  <si>
+    <t>Vic Ceder</t>
+  </si>
+  <si>
+    <t>All Headliners</t>
+  </si>
+  <si>
+    <t>GCA Callers</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -235,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -243,6 +313,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="19" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,318 +654,318 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="4" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
@@ -900,112 +973,485 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="7" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2">
+        <v>2.75</v>
+      </c>
+      <c r="C2">
+        <v>2.75</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4">
+        <v>3.5</v>
+      </c>
+      <c r="C4">
+        <v>3.5</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="3">
+        <v>16.25</v>
+      </c>
+      <c r="C5" s="3">
+        <v>16.25</v>
+      </c>
+      <c r="D5" s="3">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3">
+        <v>3</v>
+      </c>
+      <c r="G5" s="3">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="4">
+        <v>46245.56872685185</v>
+      </c>
+      <c r="C7" s="5">
+        <v>46245.56872685185</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="4">
+        <f>NOW()</f>
+        <v>46245.56872685185</v>
+      </c>
+      <c r="C8" s="5">
+        <f>NOW()</f>
+        <v>46245.56872685185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" t="str">
+        <f>IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
+        <v>✓ Up to date as of Saved</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>0.5</v>
+      </c>
+      <c r="I2">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="3">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3">
+        <v>2</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I5" s="3">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="4">
+        <v>46245.56872685185</v>
+      </c>
+      <c r="C7" s="5">
+        <v>46245.56872685185</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="4">
+        <f>NOW()</f>
+        <v>46245.56872685185</v>
+      </c>
+      <c r="C8" s="5">
+        <f>NOW()</f>
+        <v>46245.56872685185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" t="str">
+        <f>IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
+        <v>✓ Up to date as of Saved</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Shift Friday registration/GCA earlier and add a C4 slot Sunday
Registration/GCA-caller-slot now start 30 min earlier (5:00/6:00pm),
which also lengthens the GCA slot itself from 30 to 60 min. Sunday
11am-12pm Columbia bumps from C3B to C4 (Rob French unchanged) — C4
registration grew enough (4->7 dancers as of Aug 17) to justify its
own slot. Both changes come from the scratch/ proposal spreadsheet;
hour totals regenerated via generate-dance-schedule-hour-tabs.ts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Ra4hDSrkdBwdUHiTwczU3
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="77">
   <si>
     <t>Time</t>
   </si>
@@ -38,13 +38,13 @@
     <t>Columbia</t>
   </si>
   <si>
-    <t>5:30-8:00p</t>
+    <t>5:00-8:00p</t>
   </si>
   <si>
     <t>* Registration</t>
   </si>
   <si>
-    <t>6:30-7:00p</t>
+    <t>6:00-7:00p</t>
   </si>
   <si>
     <t>A2 &amp; C1: GCA Callers</t>
@@ -183,7 +183,7 @@
 ROOMS: NONE</t>
   </si>
   <si>
-    <t>C3B : Rob French</t>
+    <t>C4 : Rob French</t>
   </si>
   <si>
     <t xml:space="preserve">A2 &amp; C1 : Closing - All Headliners
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>C3B</t>
+  </si>
+  <si>
+    <t>C4</t>
   </si>
   <si>
     <t>Total</t>
@@ -1085,14 +1088,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="7" width="10" customWidth="1"/>
+    <col min="2" max="8" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>55</v>
       </c>
@@ -1114,16 +1117,19 @@
       <c r="G1" s="3" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B2">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -1135,12 +1141,15 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>9.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -1158,12 +1167,15 @@
         <v>2</v>
       </c>
       <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4">
         <v>3.5</v>
@@ -1178,21 +1190,24 @@
         <v>2</v>
       </c>
       <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>1</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="3">
-        <v>16.25</v>
+        <v>16.5</v>
       </c>
       <c r="C5" s="3">
-        <v>16.25</v>
+        <v>16.5</v>
       </c>
       <c r="D5" s="3">
         <v>15</v>
@@ -1201,39 +1216,42 @@
         <v>12</v>
       </c>
       <c r="F5" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" s="3">
-        <v>62.5</v>
+        <v>1</v>
+      </c>
+      <c r="H5" s="3">
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" s="4">
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
       <c r="C7" s="5">
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B8" s="4">
         <f>NOW()</f>
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
       <c r="C8" s="5">
         <f>NOW()</f>
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9" t="str">
         <f>IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
@@ -1242,7 +1260,7 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1272,33 +1290,33 @@
         <v>55</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1319,15 +1337,15 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>9.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -1356,7 +1374,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1385,7 +1403,7 @@
     </row>
     <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="3">
         <v>12</v>
@@ -1406,39 +1424,39 @@
         <v>2</v>
       </c>
       <c r="H5" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I5" s="3">
-        <v>62.5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" s="4">
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
       <c r="C7" s="5">
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B8" s="4">
         <f>NOW()</f>
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
       <c r="C8" s="5">
         <f>NOW()</f>
-        <v>46245.56872685185</v>
+        <v>46255.6171875</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9" t="str">
         <f>IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
@@ -1447,7 +1465,7 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Split Friday's opening slot between two callers, and show every caller regardless of hours
Splitting the 6-7pm GCA slot into two named 30-minute callers (Rob Page,
Kurt Gollhardt) exposed a bug: the Caller Schedule page required a
caller's event-wide total to exceed 3 hours before showing them a column
at all, so a short one-off session silently vanished instead of just
being a small column. Removed that threshold entirely — every real,
named caller now gets a column. The "Hours by Caller" debug/dump summary
table keeps its own, separate 3-hour floor unaffected.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DKyGwVZXVzA8t1i9DocaXZ
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -1,24 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30265F0E-CB48-5243-AB0C-D43DF9C3B1CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Friday October 9" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Saturday October 10" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Sunday October 11" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="- Hours by Level" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="- Hours by Caller" state="visible" r:id="rId8"/>
+    <sheet name="Friday October 9" sheetId="1" r:id="rId1"/>
+    <sheet name="Saturday October 10" sheetId="2" r:id="rId2"/>
+    <sheet name="Sunday October 11" sheetId="3" r:id="rId3"/>
+    <sheet name="- Hours by Level" sheetId="4" r:id="rId4"/>
+    <sheet name="- Hours by Caller" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="79">
   <si>
     <t>Time</t>
   </si>
@@ -44,19 +58,13 @@
     <t>* Registration</t>
   </si>
   <si>
-    <t>6:00-7:00p</t>
-  </si>
-  <si>
-    <t>A2 &amp; C1: GCA Callers</t>
-  </si>
-  <si>
     <t>"</t>
   </si>
   <si>
     <t>7:00p-8:00p</t>
   </si>
   <si>
-    <t xml:space="preserve">A2 &amp; C1: Trail-In Dance - All Headliners
+    <t>A2 &amp; C1: Trail-In Dance - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
   <si>
@@ -132,7 +140,7 @@
     <t>12:00p-1:00p</t>
   </si>
   <si>
-    <t xml:space="preserve">* Lunch Break (on your own)
+    <t>* Lunch Break (on your own)
 ROOMS: NONE</t>
   </si>
   <si>
@@ -163,7 +171,7 @@
     <t>5:00p-7:00p</t>
   </si>
   <si>
-    <t xml:space="preserve">* Dinner Break (on your own)
+    <t>* Dinner Break (on your own)
 ROOMS: NONE</t>
   </si>
   <si>
@@ -179,14 +187,14 @@
     <t>9:00a-11:00a</t>
   </si>
   <si>
-    <t xml:space="preserve">* Brunch in Lobby
+    <t>* Brunch in Lobby
 ROOMS: NONE</t>
   </si>
   <si>
     <t>C4 : Rob French</t>
   </si>
   <si>
-    <t xml:space="preserve">A2 &amp; C1 : Closing - All Headliners
+    <t>A2 &amp; C1 : Closing - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
   <si>
@@ -254,32 +262,46 @@
   </si>
   <si>
     <t>GCA Callers</t>
+  </si>
+  <si>
+    <t>6:00-6:30p</t>
+  </si>
+  <si>
+    <t>6:30-7:00p</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1: Rob Page</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1: Kurt Gollhardt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -657,15 +679,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -685,7 +707,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -697,81 +719,95 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>9</v>
+        <v>77</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -788,208 +824,208 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B5" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="2" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1009,121 +1045,120 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="8" width="10" customWidth="1"/>
+    <col min="1" max="8" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>61</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>63</v>
       </c>
       <c r="B2">
         <v>3</v>
@@ -1147,9 +1182,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -1173,9 +1208,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B4">
         <v>3.5</v>
@@ -1199,9 +1234,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B5" s="3">
         <v>16.5</v>
@@ -1225,9 +1260,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B7" s="4">
         <v>46255.6171875</v>
@@ -1236,43 +1271,43 @@
         <v>46255.6171875</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="4">
+        <f ca="1">NOW()</f>
+        <v>46258.742110648149</v>
+      </c>
+      <c r="C8" s="5">
+        <f ca="1">NOW()</f>
+        <v>46258.742110648149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" t="str">
+        <f ca="1">IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
+        <v>⚠ Recalculated since Saved — totals may be stale, re-run the generator script</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>67</v>
-      </c>
-      <c r="B8" s="4">
-        <f>NOW()</f>
-        <v>46255.6171875</v>
-      </c>
-      <c r="C8" s="5">
-        <f>NOW()</f>
-        <v>46255.6171875</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" t="str">
-        <f>IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
-        <v>✓ Up to date as of Saved</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1285,38 +1320,38 @@
     <col min="9" max="9" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>76</v>
-      </c>
       <c r="I1" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1343,9 +1378,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -1372,9 +1407,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1401,9 +1436,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B5" s="3">
         <v>12</v>
@@ -1430,9 +1465,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B7" s="4">
         <v>46255.6171875</v>
@@ -1441,35 +1476,35 @@
         <v>46255.6171875</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="4">
+        <f ca="1">NOW()</f>
+        <v>46258.742110648149</v>
+      </c>
+      <c r="C8" s="5">
+        <f ca="1">NOW()</f>
+        <v>46258.742110648149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" t="str">
+        <f ca="1">IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
+        <v>⚠ Recalculated since Saved — totals may be stale, re-run the generator script</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>67</v>
-      </c>
-      <c r="B8" s="4">
-        <f>NOW()</f>
-        <v>46255.6171875</v>
-      </c>
-      <c r="C8" s="5">
-        <f>NOW()</f>
-        <v>46255.6171875</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" t="str">
-        <f>IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
-        <v>✓ Up to date as of Saved</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Saturday 2-3pm Columbia caller swap in MotivateToSeattle dance schedule
Audited dance-schedule.xlsx against the new source-of-truth proposal
spreadsheet: Columbia was crediting Rob French instead of Kris Jensen for
Sat 2-3pm, leaving the 5 headline callers' hours unbalanced (13/11 instead
of 12 each, per the proposal's own "12 hrs solo" note). Also commits the
proposal spreadsheet itself (content/.../scratch/) and regenerates the
auto-generated dance-schedule-dump.md to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SH9xhnTLm8L77ELSyg8Xuj
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30265F0E-CB48-5243-AB0C-D43DF9C3B1CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19909CA-6914-854C-8FBD-FC654D9B1775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="73780" yWindow="2580" windowWidth="33420" windowHeight="26920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Friday October 9" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="81">
   <si>
     <t>Time</t>
   </si>
@@ -74,9 +74,6 @@
     <t>A2 : Ray Brendzy</t>
   </si>
   <si>
-    <t>C1 : Saundra Bryant</t>
-  </si>
-  <si>
     <t>C2 : Rob French</t>
   </si>
   <si>
@@ -92,9 +89,6 @@
     <t>C1 : Ray Brendzy</t>
   </si>
   <si>
-    <t>C2 : Saundra Bryant</t>
-  </si>
-  <si>
     <t>C3A  : Rob French</t>
   </si>
   <si>
@@ -114,9 +108,6 @@
   </si>
   <si>
     <t>10:00a-11:00a</t>
-  </si>
-  <si>
-    <t>A2 : Saundra Bryant</t>
   </si>
   <si>
     <t>C1 : Rob French</t>
@@ -150,9 +141,6 @@
     <t>C1 : Vic Ceder</t>
   </si>
   <si>
-    <t>C3B : Saundra Bryant</t>
-  </si>
-  <si>
     <t>2:00p-3:00p</t>
   </si>
   <si>
@@ -175,16 +163,10 @@
 ROOMS: NONE</t>
   </si>
   <si>
-    <t>C3A   : Saundra Bryant</t>
-  </si>
-  <si>
     <t>C3A   : Ray Brendzy</t>
   </si>
   <si>
     <t>C3A   : Michael Kellogg</t>
-  </si>
-  <si>
-    <t>9:00a-11:00a</t>
   </si>
   <si>
     <t>* Brunch in Lobby
@@ -252,9 +234,6 @@
     <t>Rob French</t>
   </si>
   <si>
-    <t>Saundra Bryant</t>
-  </si>
-  <si>
     <t>Vic Ceder</t>
   </si>
   <si>
@@ -274,6 +253,33 @@
   </si>
   <si>
     <t>A2 &amp; C1: Kurt Gollhardt</t>
+  </si>
+  <si>
+    <t>C1 : Kris Jensen</t>
+  </si>
+  <si>
+    <t>C2 : Kris Jensen</t>
+  </si>
+  <si>
+    <t>A2 : Kris Jensen</t>
+  </si>
+  <si>
+    <t>C3A   : Kris Jensen</t>
+  </si>
+  <si>
+    <t>Kris Jensen</t>
+  </si>
+  <si>
+    <t>C3B : Rob French</t>
+  </si>
+  <si>
+    <t>9:00a-10:30a</t>
+  </si>
+  <si>
+    <t>10:30-11:00a</t>
+  </si>
+  <si>
+    <t>A2 &amp; C1: Rick Hawes</t>
   </si>
 </sst>
 </file>
@@ -302,6 +308,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -721,11 +728,11 @@
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>8</v>
@@ -735,11 +742,11 @@
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
@@ -765,31 +772,31 @@
         <v>12</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -826,137 +833,137 @@
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>19</v>
+        <v>73</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -964,16 +971,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -981,33 +988,33 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1018,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1047,73 +1054,84 @@
     </row>
     <row r="2" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="2"/>
+        <v>79</v>
+      </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>51</v>
+        <v>80</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="F5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>52</v>
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1132,33 +1150,33 @@
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B2">
         <v>3</v>
@@ -1184,7 +1202,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -1210,7 +1228,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B4">
         <v>3.5</v>
@@ -1236,7 +1254,7 @@
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B5" s="3">
         <v>16.5</v>
@@ -1262,7 +1280,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B7" s="4">
         <v>46255.6171875</v>
@@ -1273,20 +1291,20 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B8" s="4">
         <f ca="1">NOW()</f>
-        <v>46258.742110648149</v>
+        <v>46268.33246701389</v>
       </c>
       <c r="C8" s="5">
         <f ca="1">NOW()</f>
-        <v>46258.742110648149</v>
+        <v>46268.33246701389</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B9" t="str">
         <f ca="1">IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
@@ -1295,7 +1313,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1322,36 +1340,36 @@
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1380,7 +1398,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -1409,7 +1427,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1438,7 +1456,7 @@
     </row>
     <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B5" s="3">
         <v>12</v>
@@ -1467,7 +1485,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B7" s="4">
         <v>46255.6171875</v>
@@ -1478,20 +1496,20 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B8" s="4">
         <f ca="1">NOW()</f>
-        <v>46258.742110648149</v>
+        <v>46268.33246701389</v>
       </c>
       <c r="C8" s="5">
         <f ca="1">NOW()</f>
-        <v>46258.742110648149</v>
+        <v>46268.33246701389</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B9" t="str">
         <f ca="1">IF(C8&gt;C7+TIME(0,0,15),"⚠ Recalculated since Saved — totals may be stale, re-run the generator script","✓ Up to date as of Saved")</f>
@@ -1500,7 +1518,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
One room for Rick
</commit_message>
<xml_diff>
--- a/content/MotivateToSeattle/data/dance-schedule.xlsx
+++ b/content/MotivateToSeattle/data/dance-schedule.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26E14798-D3C6-DA4F-98B0-6E4313B5DC22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="73780" yWindow="2580" windowWidth="33420" windowHeight="26920" activeTab="2"/>
+    <workbookView xWindow="14420" yWindow="1280" windowWidth="33420" windowHeight="26920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Friday October 9" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Saturday October 10" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Sunday October 11" state="visible" r:id="rId6"/>
+    <sheet name="Friday October 9" sheetId="1" r:id="rId1"/>
+    <sheet name="Saturday October 10" sheetId="2" r:id="rId2"/>
+    <sheet name="Sunday October 11" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="59">
   <si>
     <t>Time</t>
   </si>
@@ -60,7 +61,7 @@
     <t>7:00p-8:00p</t>
   </si>
   <si>
-    <t xml:space="preserve">A2 &amp; C1: Trail-In Dance - All Headliners
+    <t>A2 &amp; C1: Trail-In Dance - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
   <si>
@@ -136,7 +137,7 @@
     <t>12:00p-1:00p</t>
   </si>
   <si>
-    <t xml:space="preserve">* Lunch Break (on your own)
+    <t>* Lunch Break (on your own)
 ROOMS: NONE</t>
   </si>
   <si>
@@ -170,7 +171,7 @@
     <t>5:00p-7:00p</t>
   </si>
   <si>
-    <t xml:space="preserve">* Dinner Break (on your own)
+    <t>* Dinner Break (on your own)
 ROOMS: NONE</t>
   </si>
   <si>
@@ -183,7 +184,7 @@
     <t>9:00a-10:30a</t>
   </si>
   <si>
-    <t xml:space="preserve">* Brunch in Lobby
+    <t>* Brunch in Lobby
 ROOMS: NONE</t>
   </si>
   <si>
@@ -196,28 +197,28 @@
     <t>C4 : Rob French</t>
   </si>
   <si>
-    <t xml:space="preserve">A2 &amp; C1 : Closing - All Headliners
+    <t>A2 &amp; C1 : Closing - All Headliners
 ROOMS: Glacier, Horizon</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -592,15 +593,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -620,7 +621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -632,7 +633,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -646,7 +647,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -660,7 +661,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -669,7 +670,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -687,7 +688,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -707,20 +708,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -737,7 +738,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
@@ -754,7 +755,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -771,7 +772,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -788,7 +789,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>38</v>
       </c>
@@ -796,7 +797,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
@@ -813,7 +814,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>43</v>
       </c>
@@ -830,7 +831,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>46</v>
       </c>
@@ -847,7 +848,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>47</v>
       </c>
@@ -864,7 +865,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>49</v>
       </c>
@@ -872,7 +873,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -889,7 +890,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
@@ -906,7 +907,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -925,20 +926,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,7 +959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>53</v>
       </c>
@@ -966,18 +967,15 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -995,7 +993,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>38</v>
       </c>
@@ -1013,7 +1011,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
@@ -1031,7 +1029,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>43</v>
       </c>
@@ -1042,6 +1040,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>